<commit_message>
Add month-close workflow so the template survives across months
「毎月シートを増やす」方式をやめ、月末の締め処理で継続運用する仕組みを追加。
ブックの枚数は月に関係なく一定になる。

- 15_KPI累積ログ: 週次KPIを値で積み上げる保管庫（対象月を切り替えても
  過去実績が消えない）
- 16_年間推移: 累積ログを月別集計した年度推移（率は週平均、件数は月合計）
- tools/pdca/close_month.py: 当月ブックを実績として保管し、週次KPIを累積ログへ
  値で追記し、日別入力を空にして対象月を進めた翌月ブックを生成。同一施設・
  同一年月の二重登録は拒否する
- 00_はじめに / 08_運用ルール / 07_改善提案一覧 に月次サイクルを追記

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LiRaWe1BqN12Rhy9y1p4p2
</commit_message>
<xml_diff>
--- a/dist/週間PDCA_改善版テンプレート.xlsx
+++ b/dist/週間PDCA_改善版テンプレート.xlsx
@@ -22,6 +22,8 @@
     <sheet name="12_月次_営業行動" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_月次_加算要件" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="14_案件管理台帳" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15_KPI累積ログ" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="16_年間推移" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="施設名リスト">'01_施設マスタ'!$B$2:$B$41</definedName>
@@ -35,8 +37,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_施設マスタ'!$A$1:$I$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_課題管理表'!$A$1:$U$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_週次KPIログ'!$A$1:$P$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_改善提案一覧'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_改善提案一覧'!$A$1:$G$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'14_案件管理台帳'!$A$1:$Q$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'15_KPI累積ログ'!$A$1:$P$2000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -610,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C11"/>
+  <dimension ref="B2:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -707,10 +710,34 @@
     <row r="11" ht="34" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>継続運用</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>月ごとにシートを増やしません。月末に締め処理を行うと、当月ブックが実績として保管され、週次KPIは 15_KPI累積ログ に値で積み上がり、日別入力欄が空の翌月ブックが作られます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>過去の参照</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>月をまたいだ推移は 16_年間推移 で見ます。個別の日別実績は、締めのときに保管された『〇〇_実績.xlsx』を開いてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>改善の根拠</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>07_改善提案一覧 に、旧シートで検出した具体的な不具合と改善内容を記載しています。</t>
         </is>
@@ -9127,6 +9154,854 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>記録日</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>対象施設</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>年</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>週</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>カテゴリ</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>指標名</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>週次目標</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>実績</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>達成率</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>差異</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>担当者</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>未達要因（Check）</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>次週アクション（Act）</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>締め処理日</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="R3" s="28" t="inlineStr">
+        <is>
+          <t>このシートは月締め処理（tools/pdca/close_month.py）で自動追記される保管庫です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="R4" s="13" t="inlineStr">
+        <is>
+          <t>・数式ではなく『値』が入ります。対象月を切り替えても過去の実績が消えません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t>・手で編集しないでください。修正が必要な場合は該当行を直し、締め日を入れ直します。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="R6" s="13" t="inlineStr">
+        <is>
+          <t>・40施設分をこのシートに縦に積めば、そのままピボットで全社集計できます。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P2000"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:P15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>年間推移（15_KPI累積ログの集計）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="20">
+        <f>設定対象年&amp;"年度／"&amp;設定対象施設</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>※ 月締めが済んだ月だけ数値が入ります。率は週平均、件数は月合計です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>指標名</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>4月</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>5月</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>6月</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>7月</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>8月</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>9月</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>10月</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>11月</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>1月</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>2月</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>3月</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>年度計/平均</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>GH稼働率</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B7,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="17">
+        <f>IFERROR(AVERAGE($D7:$O7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>営業接点件数</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B8,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P8" s="4">
+        <f>IFERROR(SUM($D8:$O8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>見学・体験件数</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B9,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P9" s="4">
+        <f>IFERROR(SUM($D9:$O9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>入居契約件数</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B10,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="4">
+        <f>IFERROR(SUM($D10:$O10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SS稼働率</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B11,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="17">
+        <f>IFERROR(AVERAGE($D11:$O11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>SS案件発掘件数</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B12,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="4">
+        <f>IFERROR(SUM($D12:$O12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>夜勤加配 取得率</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="17">
+        <f>IFERROR(AVERAGEIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B13,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="17">
+        <f>IFERROR(AVERAGE($D13:$O13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>訪看契約件数</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B14,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="4">
+        <f>IFERROR(SUM($D14:$O14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SQ契約件数</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="D15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,4),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,5),"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,6),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,7),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,8),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,9),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,10),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,11),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年,'15_KPI累積ログ'!$D$2:$D$2000,12),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,1),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,2),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="4">
+        <f>IFERROR(SUMIFS('15_KPI累積ログ'!$J$2:$J$2000,'15_KPI累積ログ'!$G$2:$G$2000,$B15,'15_KPI累積ログ'!$C$2:$C$2000,設定対象年+1,'15_KPI累積ログ'!$D$2:$D$2000,3),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="4">
+        <f>IFERROR(SUM($D15:$O15),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -17650,7 +18525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17950,27 +18825,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>運用</t>
+          <t>構造</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>対応方針・所感が1セルに改行で詰め込まれた長文（【営業行動】…▶2/25 追客 等）。</t>
+          <t>継続運用の方法が『月シートを1枚ずつ増やす』こと。実ファイルでは22枚まで増え、命名も不統一になっている。</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>目標値と実績が数式で取り出せず、達成／未達の自動判定ができない。読む人によって解釈が変わる。</t>
+          <t>シートが増えるほどブックが重くなり、集計式（12か月固定のHLOOKUP表）が追従できない。年度をまたぐと参照が壊れ、過去の修正が現在の集計に波及する。</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>『数値で置く欄』と『文章で残す欄』を分離する。</t>
+          <t>月ごとにシートを増やさず、月末に締めて『実績ブックの保管＋累積ログへの追記＋翌月ブックの生成』に分ける。</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>週次目標・実績・達成率・差異を数値列に分離し、所感は別列に残す。</t>
+          <t>15_KPI累積ログ（値で保管）＋16_年間推移＋tools/pdca/close_month.py（締め処理）。ブックの枚数は月に関係なく一定。</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -17990,22 +18865,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>ステータス列・期限列（G/H, P/Q…）は結合セルで、入力規則も条件付き書式もなく空欄のまま。</t>
+          <t>対応方針・所感が1セルに改行で詰め込まれた長文（【営業行動】…▶2/25 追客 等）。</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>期限超過が誰にも見えない。ステータスの表記ゆれ（完了／済／OK）で集計不能。</t>
+          <t>目標値と実績が数式で取り出せず、達成／未達の自動判定ができない。読む人によって解釈が変わる。</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>ステータスはプルダウン、期限は日付、遅延は自動判定＋色付け。</t>
+          <t>『数値で置く欄』と『文章で残す欄』を分離する。</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>04_課題管理表にステータスDV・残日数・遅延判定・行の自動着色を実装。</t>
+          <t>週次目標・実績・達成率・差異を数値列に分離し、所感は別列に残す。</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -18025,27 +18900,27 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>『※未対象施設』とだけ書かれた行（④訪看契約・⑤SQ利用）が毎週コピーされ続けている。</t>
+          <t>ステータス列・期限列（G/H, P/Q…）は結合セルで、入力規則も条件付き書式もなく空欄のまま。</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>対象外の項目が常時表示され、シートのノイズになる。対象化した時に誰が判断するか決まっていない。</t>
+          <t>期限超過が誰にも見えない。ステータスの表記ゆれ（完了／済／OK）で集計不能。</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>対象／対象外を施設マスタ側の属性で持ち、非対象は非表示にする。</t>
+          <t>ステータスはプルダウン、期限は日付、遅延は自動判定＋色付け。</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>01_施設マスタ I列『PDCA対象』で管理。カテゴリは04で必要な行だけ起票する運用。</t>
+          <t>04_課題管理表にステータスDV・残日数・遅延判定・行の自動着色を実装。</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
     </row>
@@ -18060,22 +18935,22 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>『週間PDCA (見本)』が本体と別に存在し、内容が本体とずれている。</t>
+          <t>『※未対象施設』とだけ書かれた行（④訪看契約・⑤SQ利用）が毎週コピーされ続けている。</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>見本の更新漏れで、書き方の基準が人によって変わる。</t>
+          <t>対象外の項目が常時表示され、シートのノイズになる。対象化した時に誰が判断するか決まっていない。</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>見本を別シートで持たず、テンプレート自体に入力例と注記を持たせる。</t>
+          <t>対象／対象外を施設マスタ側の属性で持ち、非対象は非表示にする。</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>00_はじめに に運用手順、各シートの黄色セルで入力箇所を明示。</t>
+          <t>01_施設マスタ I列『PDCA対象』で管理。カテゴリは04で必要な行だけ起票する運用。</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -18095,22 +18970,22 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>予算達成状況の判定が =IF(予算比&gt;=0,"〇","✕") の2値のみ。前月比の一部は文字列 '-'。</t>
+          <t>『週間PDCA (見本)』が本体と別に存在し、内容が本体とずれている。</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>あと一歩の未達と大幅未達が同じ『✕』。文字列混在で平均・グラフが崩れる。</t>
+          <t>見本の更新漏れで、書き方の基準が人によって変わる。</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>達成／要注意／未達の3段階にし、空欄は空欄のまま扱う。</t>
+          <t>見本を別シートで持たず、テンプレート自体に入力例と注記を持たせる。</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>06_ダッシュボードで 100%以上=〇、90%以上=△、それ未満=✕、未入力は『未入力』と判定。</t>
+          <t>00_はじめに に運用手順、各シートの黄色セルで入力箇所を明示。</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -18125,27 +19000,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>データ</t>
+          <t>運用</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Sheet2 に居室番号・区分・年齢の生データが残置。個人に紐づく情報がシート内に混在。</t>
+          <t>予算達成状況の判定が =IF(予算比&gt;=0,"〇","✕") の2値のみ。前月比の一部は文字列 '-'。</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>配布時に意図しない情報が同梱される。マスタとしての位置づけも不明。</t>
+          <t>あと一歩の未達と大幅未達が同じ『✕』。文字列混在で平均・グラフが崩れる。</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>個人データは配布用テンプレートから分離する。</t>
+          <t>達成／要注意／未達の3段階にし、空欄は空欄のまま扱う。</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>本テンプレートには個人データを含めない。必要なら別ファイルで管理。</t>
+          <t>06_ダッシュボードで 100%以上=〇、90%以上=△、それ未満=✕、未入力は『未入力』と判定。</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -18160,27 +19035,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>拡張</t>
+          <t>データ</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>施設一覧側に『グループホームイノベル信中島／公式名 小信中島』など名称差3件、住所照合注記あり。</t>
+          <t>Sheet2 に居室番号・区分・年齢の生データが残置。個人に紐づく情報がシート内に混在。</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>施設名がキーなのに正式名称と社内呼称が混在すると、集計時に名寄せできない。</t>
+          <t>配布時に意図しない情報が同梱される。マスタとしての位置づけも不明。</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>施設IDを主キーにし、名称は表示用の属性として持つ。</t>
+          <t>個人データは配布用テンプレートから分離する。</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>01_施設マスタに施設ID（F001〜F040）を付与。名称変更はマスタ1か所で吸収。</t>
+          <t>本テンプレートには個人データを含めない。必要なら別ファイルで管理。</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -18195,32 +19070,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>構造</t>
+          <t>拡張</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>月シート（4月〜26年9月の22枚）が、利用者ごとの日別稼働カレンダー・SS予約・営業行動・案件管理・加算要件の入力面を兼ねている。週間PDCAの文章は BF16 等の長大な文字列連結式で自動生成されている。</t>
+          <t>施設一覧側に『グループホームイノベル信中島／公式名 小信中島』など名称差3件、住所照合注記あり。</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>入力面（原簿）と管理面（PDCA）が同じシートに同居し、月が変わるたびシートを増やす必要がある。連結式で作った文章は、あとから数値として再利用できない。</t>
+          <t>施設名がキーなのに正式名称と社内呼称が混在すると、集計時に名寄せできない。</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>原簿は月次入力シートとして分離し、集計値だけをPDCA側へ渡す。</t>
+          <t>施設IDを主キーにし、名称は表示用の属性として持つ。</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>10〜13の月次入力シートに分離。週別集計値は05_週次KPIログが自動で参照する。</t>
+          <t>01_施設マスタに施設ID（F001〜F040）を付与。名称変更はマスタ1か所で吸収。</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
     </row>
@@ -18235,22 +19110,22 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>案件管理が『kintone名×日別セルに進捗記号』のマトリクス（55〜78行）。相談元・区分・希望種別が別セルに散る。</t>
+          <t>月シート（4月〜26年9月の22枚）が、利用者ごとの日別稼働カレンダー・SS予約・営業行動・案件管理・加算要件の入力面を兼ねている。週間PDCAの文章は BF16 等の長大な文字列連結式で自動生成されている。</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>同じ案件の履歴が月シートをまたいで分断され、発掘→見学→体験→契約のリードタイムが測れない。</t>
+          <t>入力面（原簿）と管理面（PDCA）が同じシートに同居し、月が変わるたびシートを増やす必要がある。連結式で作った文章は、あとから数値として再利用できない。</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>案件は1件1行の台帳にし、各フェーズの日付を列で持つ。</t>
+          <t>原簿は月次入力シートとして分離し、集計値だけをPDCA側へ渡す。</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>14_案件管理台帳。日付列から見学・体験・入居件数を週次で自動集計し、停滞14日超は赤表示。</t>
+          <t>10〜13の月次入力シートに分離。週別集計値は05_週次KPIログが自動で参照する。</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -18265,32 +19140,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>運用</t>
+          <t>構造</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>重度障害者支援体制・福祉専門職員配置等加算の要件確認が、月シートの隅にチェック欄として置かれている（BR88 常勤比率0.368→✕ 等）。</t>
+          <t>案件管理が『kintone名×日別セルに進捗記号』のマトリクス（55〜78行）。相談元・区分・希望種別が別セルに散る。</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>算定可否の根拠が月シートを開かないと見えず、要件を割った時に誰がいつ気づくかが運用任せ。</t>
+          <t>同じ案件の履歴が月シートをまたいで分断され、発掘→見学→体験→契約のリードタイムが測れない。</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>要件判定を独立させ、割り込み時に『要対応』として表示する。</t>
+          <t>案件は1件1行の台帳にし、各フェーズの日付を列で持つ。</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>13_月次_加算要件に集約。夜勤加配は日別実績から取得率を自動計算、体制加算は✕が1つでもあれば『要対応』。</t>
+          <t>14_案件管理台帳。日付列から見学・体験・入居件数を週次で自動集計し、停滞14日超は赤表示。</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
     </row>
@@ -18300,38 +19175,73 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t>運用</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>重度障害者支援体制・福祉専門職員配置等加算の要件確認が、月シートの隅にチェック欄として置かれている（BR88 常勤比率0.368→✕ 等）。</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>算定可否の根拠が月シートを開かないと見えず、要件を割った時に誰がいつ気づくかが運用任せ。</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>要件判定を独立させ、割り込み時に『要対応』として表示する。</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>13_月次_加算要件に集約。夜勤加配は日別実績から取得率を自動計算、体制加算は✕が1つでもあれば『要対応』。</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>拡張</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>40施設分のファイルが個別に存在し、AMは自分の担当分だけを見る運用。</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>エリア長・本部が全体傾向（未達KPI・遅延課題の偏り）を把握するのに手作業の集約が必要。</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>縦持ちログを束ねてピボット集計できる形にする。</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>05_週次KPIログは施設名・担当者を各行に持つため、40施設分を連結してそのまま集計可能。06に担当AM別の遅延件数を実装。</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>中</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G19"/>
-  <conditionalFormatting sqref="G2:G19">
+  <autoFilter ref="A1:G20"/>
+  <conditionalFormatting sqref="G2:G20">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$G2="高"</formula>
     </cfRule>
@@ -18346,7 +19256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E10"/>
+  <dimension ref="B2:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -18498,20 +19408,64 @@
     <row r="10" ht="30" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>月次（月末）</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>担当AM</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Excelで保存後、月締め処理を実行して翌月ブックを作成</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>締める前に必ずExcelで保存する（数式の値が確定するため）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>月次（翌月初）</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>担当AM</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>16_年間推移で前月までの推移を確認</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>2か月連続で未達のKPIは対応方針を作り直す</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>随時</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>本部</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>01_施設マスタの担当変更・新規開設を反映</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>マスタ更新は本部のみ。現場は編集しない</t>
         </is>

</xml_diff>